<commit_message>
update ML-prescription (#131) ed5577d23fe75d42b5cdc2397c8fcc13858cf058
</commit_message>
<xml_diff>
--- a/fusionModeleLogique/ig/StructureDefinition-fr-lm-administration-blood-derivatives.xlsx
+++ b/fusionModeleLogique/ig/StructureDefinition-fr-lm-administration-blood-derivatives.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-24T13:15:59+00:00</t>
+    <t>2026-04-29T08:17:29+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -269,11 +269,11 @@
     <t>fr-lm-administration-blood-derivatives.header.subject</t>
   </si>
   <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-lm-patient-usager
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-lm-patient
 </t>
   </si>
   <si>
-    <t>Patient/subject information</t>
+    <t>Patient / Usager</t>
   </si>
   <si>
     <t>fr-lm-entry.header.subject</t>
@@ -443,7 +443,7 @@
     <t>fr-lm-entry.header.source</t>
   </si>
   <si>
-    <t>fr-lm-administration-blood-derivatives.header.langue</t>
+    <t>fr-lm-administration-blood-derivatives.header.language</t>
   </si>
   <si>
     <t>'fr-FR' pour français métropolitain (la casse des caractères doit être respectée)
@@ -451,7 +451,7 @@
 La partie en majuscules indique le code pays (ISO-3166)</t>
   </si>
   <si>
-    <t>fr-lm-entry.header.langue</t>
+    <t>fr-lm-entry.header.language</t>
   </si>
   <si>
     <t>fr-lm-administration-blood-derivatives.code</t>

</xml_diff>

<commit_message>
Mise à jour du status 13678e2faadb781f6b21fa351ea532ec73372b19
</commit_message>
<xml_diff>
--- a/fusionModeleLogique/ig/StructureDefinition-fr-lm-administration-blood-derivatives.xlsx
+++ b/fusionModeleLogique/ig/StructureDefinition-fr-lm-administration-blood-derivatives.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="693" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="693" uniqueCount="145">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-29T08:17:29+00:00</t>
+    <t>2026-04-29T08:41:15+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -422,13 +422,7 @@
 </t>
   </si>
   <si>
-    <t>Statut de l'acte</t>
-  </si>
-  <si>
-    <t>jdv-hl7-v3-ActStatus-cisis (2.16.840.1.113883.1.11.15933)</t>
-  </si>
-  <si>
-    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-hl7-v3-ActStatus-cisis</t>
+    <t>Statut</t>
   </si>
   <si>
     <t>fr-lm-entry.header.status</t>
@@ -796,8 +790,8 @@
     <col min="22" max="22" width="15.13671875" customWidth="true" bestFit="true"/>
     <col min="23" max="23" width="16.3203125" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="16.16796875" customWidth="true" bestFit="true"/>
-    <col min="25" max="25" width="47.0546875" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="52.58203125" customWidth="true" bestFit="true"/>
+    <col min="25" max="25" width="18.49609375" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="16.828125" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="17.65625" customWidth="true" bestFit="true"/>
@@ -2432,7 +2426,7 @@
       </c>
       <c r="E17" s="2"/>
       <c r="F17" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="G17" t="s" s="2">
         <v>79</v>
@@ -2483,31 +2477,31 @@
         <v>73</v>
       </c>
       <c r="Y17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF17" t="s" s="2">
         <v>133</v>
       </c>
-      <c r="Z17" t="s" s="2">
-        <v>134</v>
-      </c>
-      <c r="AA17" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AB17" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AC17" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AD17" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AE17" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AF17" t="s" s="2">
-        <v>135</v>
-      </c>
       <c r="AG17" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="AH17" t="s" s="2">
         <v>79</v>
@@ -2521,10 +2515,10 @@
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
@@ -2550,10 +2544,10 @@
         <v>131</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="M18" t="s" s="2">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
@@ -2604,7 +2598,7 @@
         <v>73</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>74</v>
@@ -2621,10 +2615,10 @@
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
@@ -2650,10 +2644,10 @@
         <v>131</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
@@ -2704,7 +2698,7 @@
         <v>73</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>74</v>
@@ -2721,10 +2715,10 @@
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
@@ -2750,10 +2744,10 @@
         <v>131</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
@@ -2804,7 +2798,7 @@
         <v>73</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>79</v>
@@ -2821,10 +2815,10 @@
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -2847,13 +2841,13 @@
         <v>73</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
@@ -2904,7 +2898,7 @@
         <v>73</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>79</v>

</xml_diff>